<commit_message>
feat: initialize and add weight matrices for v1.8, v1.8.1, and v3.1 model versions
</commit_message>
<xml_diff>
--- a/version1.xlsx
+++ b/version1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jim94\Documents\numberAI\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6D29FABA-A2DD-4B46-BCB7-AD2FFFDBF0DB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D02BF22A-91B9-4B01-A31D-BCDD47B1031B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{6637884C-02A6-4E8C-9587-F36CA748A09F}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="20">
   <si>
     <t>version</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -118,10 +118,6 @@
   </si>
   <si>
     <t>N/A</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>32 #</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -531,7 +527,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F3D1C9E5-31F4-41BB-833E-D7E3F68487BE}">
-  <dimension ref="A1:Q17"/>
+  <dimension ref="A1:Q24"/>
   <sheetFormatPr defaultRowHeight="15.4" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="8" width="9.06640625" style="2"/>
@@ -642,11 +638,11 @@
       </c>
       <c r="G3" s="1"/>
       <c r="M3" s="2">
-        <f t="shared" ref="M3:M17" si="0">C3*D3</f>
+        <f t="shared" ref="M3:M29" si="0">C3*D3</f>
         <v>8192</v>
       </c>
       <c r="N3" s="2">
-        <f t="shared" ref="N3:N17" si="1">E3*F3</f>
+        <f t="shared" ref="N3:N24" si="1">E3*F3</f>
         <v>320</v>
       </c>
       <c r="O3" s="2">
@@ -714,8 +710,8 @@
       <c r="D5" s="1">
         <v>16</v>
       </c>
-      <c r="E5" s="3" t="s">
-        <v>20</v>
+      <c r="E5" s="3">
+        <v>32</v>
       </c>
       <c r="F5" s="1">
         <v>10</v>
@@ -731,17 +727,17 @@
         <f t="shared" si="0"/>
         <v>4096</v>
       </c>
-      <c r="N5" s="2" t="e">
-        <f t="shared" si="1"/>
-        <v>#VALUE!</v>
+      <c r="N5" s="2">
+        <f t="shared" si="1"/>
+        <v>320</v>
       </c>
       <c r="O5" s="2">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="P5" s="2" t="e">
+      <c r="P5" s="2">
         <f t="shared" si="3"/>
-        <v>#VALUE!</v>
+        <v>4416</v>
       </c>
       <c r="Q5" s="2">
         <v>92.03</v>
@@ -1158,7 +1154,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:15" x14ac:dyDescent="0.45">
+    <row r="17" spans="1:17" x14ac:dyDescent="0.45">
       <c r="A17" s="4"/>
       <c r="B17" s="4"/>
       <c r="C17" s="1">
@@ -1182,6 +1178,137 @@
       </c>
       <c r="O17" s="2">
         <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" spans="1:17" x14ac:dyDescent="0.45">
+      <c r="A18" s="2">
+        <v>1.8</v>
+      </c>
+      <c r="B18" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C18" s="2">
+        <v>784</v>
+      </c>
+      <c r="D18" s="2">
+        <v>28</v>
+      </c>
+      <c r="E18" s="2">
+        <v>196</v>
+      </c>
+      <c r="F18" s="2">
+        <v>10</v>
+      </c>
+      <c r="M18" s="2">
+        <f t="shared" si="0"/>
+        <v>21952</v>
+      </c>
+      <c r="N18" s="2">
+        <f t="shared" si="1"/>
+        <v>1960</v>
+      </c>
+      <c r="P18" s="2">
+        <f>SUM(M18:N24)</f>
+        <v>24416</v>
+      </c>
+      <c r="Q18" s="2">
+        <v>95.14</v>
+      </c>
+    </row>
+    <row r="19" spans="1:17" x14ac:dyDescent="0.45">
+      <c r="C19" s="2">
+        <v>28</v>
+      </c>
+      <c r="D19" s="2">
+        <v>4</v>
+      </c>
+      <c r="M19" s="2">
+        <f t="shared" si="0"/>
+        <v>112</v>
+      </c>
+      <c r="N19" s="2">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" spans="1:17" x14ac:dyDescent="0.45">
+      <c r="C20" s="2">
+        <v>28</v>
+      </c>
+      <c r="D20" s="2">
+        <v>4</v>
+      </c>
+      <c r="M20" s="2">
+        <f t="shared" si="0"/>
+        <v>112</v>
+      </c>
+      <c r="N20" s="2">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" spans="1:17" x14ac:dyDescent="0.45">
+      <c r="C21" s="2">
+        <v>28</v>
+      </c>
+      <c r="D21" s="2">
+        <v>4</v>
+      </c>
+      <c r="M21" s="2">
+        <f t="shared" si="0"/>
+        <v>112</v>
+      </c>
+      <c r="N21" s="2">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22" spans="1:17" x14ac:dyDescent="0.45">
+      <c r="C22" s="2">
+        <v>28</v>
+      </c>
+      <c r="D22" s="2">
+        <v>4</v>
+      </c>
+      <c r="M22" s="2">
+        <f t="shared" si="0"/>
+        <v>112</v>
+      </c>
+      <c r="N22" s="2">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23" spans="1:17" x14ac:dyDescent="0.45">
+      <c r="C23" s="2">
+        <v>14</v>
+      </c>
+      <c r="D23" s="2">
+        <v>2</v>
+      </c>
+      <c r="M23" s="2">
+        <f t="shared" si="0"/>
+        <v>28</v>
+      </c>
+      <c r="N23" s="2">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24" spans="1:17" x14ac:dyDescent="0.45">
+      <c r="C24" s="2">
+        <v>14</v>
+      </c>
+      <c r="D24" s="2">
+        <v>2</v>
+      </c>
+      <c r="M24" s="2">
+        <f t="shared" si="0"/>
+        <v>28</v>
+      </c>
+      <c r="N24" s="2">
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>

</xml_diff>